<commit_message>
updated the external links.
</commit_message>
<xml_diff>
--- a/VT_REG1_ELC_V12.xlsx
+++ b/VT_REG1_ELC_V12.xlsx
@@ -1,27 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" mc:Ignorable="x15 xr xr6 xr10">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22730"/>
-  <workbookPr showObjects="placeholders" codeName="ThisWorkbook"/>
+  <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\VEDA\Training material\DemoS_012\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8F285464-C26D-4EE5-8AAA-6C1B248B09E6}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1905" yWindow="1905" windowWidth="21600" windowHeight="11385" tabRatio="901" activeTab="3"/>
   </bookViews>
   <sheets>
-    <sheet name="EB1" sheetId="133" r:id="rId1"/>
-    <sheet name="RES_ELC" sheetId="152" r:id="rId2"/>
-    <sheet name="Sector_Fuels_ELC" sheetId="140" r:id="rId3"/>
-    <sheet name="Con_ELC" sheetId="143" r:id="rId4"/>
-    <sheet name="Emi" sheetId="149" r:id="rId5"/>
+    <sheet name="EB1" sheetId="133" r:id="rId3"/>
+    <sheet name="RES_ELC" sheetId="152" r:id="rId4"/>
+    <sheet name="Sector_Fuels_ELC" sheetId="140" r:id="rId5"/>
+    <sheet name="Con_ELC" sheetId="143" r:id="rId6"/>
+    <sheet name="Emi" sheetId="149" r:id="rId7"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId6"/>
-    <externalReference r:id="rId7"/>
+    <externalReference r:id="rId9"/>
+    <externalReference r:id="rId10"/>
   </externalReferences>
   <definedNames>
     <definedName name="FID_1">[1]AGR_Fuels!$A$2</definedName>
@@ -38,20 +37,19 @@
 </workbook>
 </file>
 
-<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>Gary Goldstein</author>
     <author>Amit Kanudia</author>
     <author>Maurizio Gargiulo</author>
   </authors>
   <commentList>
-    <comment ref="J3" authorId="0" shapeId="0">
+    <comment ref="J3" authorId="0">
       <text>
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -63,7 +61,6 @@
           <rPr>
             <b/>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -72,7 +69,6 @@
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -83,7 +79,6 @@
           <rPr>
             <b/>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -92,7 +87,6 @@
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -103,7 +97,6 @@
           <rPr>
             <b/>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -112,7 +105,6 @@
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -123,7 +115,6 @@
           <rPr>
             <b/>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -132,7 +123,6 @@
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -143,7 +133,6 @@
           <rPr>
             <b/>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -152,7 +141,6 @@
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -160,13 +148,12 @@
         </r>
       </text>
     </comment>
-    <comment ref="O3" authorId="1" shapeId="0">
+    <comment ref="O3" authorId="1">
       <text>
         <r>
           <rPr>
             <b/>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -175,7 +162,6 @@
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -186,12 +172,11 @@
         </r>
       </text>
     </comment>
-    <comment ref="P3" authorId="2" shapeId="0">
+    <comment ref="P3" authorId="2">
       <text>
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -201,7 +186,6 @@
           <rPr>
             <b/>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -211,7 +195,6 @@
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -221,7 +204,6 @@
           <rPr>
             <b/>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -231,7 +213,6 @@
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -241,7 +222,6 @@
           <rPr>
             <b/>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -251,7 +231,6 @@
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -259,12 +238,11 @@
         </r>
       </text>
     </comment>
-    <comment ref="Q3" authorId="2" shapeId="0">
+    <comment ref="Q3" authorId="2">
       <text>
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -274,7 +252,6 @@
           <rPr>
             <b/>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -284,7 +261,6 @@
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -294,7 +270,6 @@
           <rPr>
             <b/>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -304,7 +279,6 @@
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -312,12 +286,11 @@
         </r>
       </text>
     </comment>
-    <comment ref="R3" authorId="2" shapeId="0">
+    <comment ref="R3" authorId="2">
       <text>
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -328,7 +301,6 @@
           <rPr>
             <b/>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -337,7 +309,6 @@
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -345,12 +316,11 @@
         </r>
       </text>
     </comment>
-    <comment ref="P15" authorId="2" shapeId="0">
+    <comment ref="P15" authorId="2">
       <text>
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -361,7 +331,6 @@
           <rPr>
             <b/>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -370,7 +339,6 @@
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -381,7 +349,6 @@
           <rPr>
             <b/>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -390,7 +357,6 @@
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -401,7 +367,6 @@
           <rPr>
             <b/>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -410,7 +375,6 @@
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -421,7 +385,6 @@
           <rPr>
             <b/>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -430,7 +393,6 @@
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -438,13 +400,12 @@
         </r>
       </text>
     </comment>
-    <comment ref="Q15" authorId="1" shapeId="0">
+    <comment ref="Q15" authorId="1">
       <text>
         <r>
           <rPr>
             <b/>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -453,7 +414,6 @@
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -463,12 +423,11 @@
         </r>
       </text>
     </comment>
-    <comment ref="R15" authorId="2" shapeId="0">
+    <comment ref="R15" authorId="2">
       <text>
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -478,7 +437,6 @@
           <rPr>
             <b/>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -488,7 +446,6 @@
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -498,7 +455,6 @@
           <rPr>
             <b/>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -507,7 +463,6 @@
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -517,7 +472,6 @@
           <rPr>
             <b/>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -526,12 +480,11 @@
         </r>
       </text>
     </comment>
-    <comment ref="J16" authorId="2" shapeId="0">
+    <comment ref="J16" authorId="2">
       <text>
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -540,7 +493,6 @@
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -551,7 +503,6 @@
           <rPr>
             <b/>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -561,7 +512,6 @@
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -571,7 +521,6 @@
           <rPr>
             <b/>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -581,7 +530,6 @@
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -591,7 +539,6 @@
           <rPr>
             <b/>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -601,7 +548,6 @@
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -611,7 +557,6 @@
           <rPr>
             <b/>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -621,7 +566,6 @@
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -631,7 +575,6 @@
           <rPr>
             <b/>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -641,7 +584,6 @@
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -651,7 +593,6 @@
           <rPr>
             <b/>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -661,7 +602,6 @@
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -671,7 +611,6 @@
           <rPr>
             <b/>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -681,7 +620,6 @@
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -692,7 +630,6 @@
           <rPr>
             <b/>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -701,7 +638,6 @@
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -711,7 +647,6 @@
           <rPr>
             <b/>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -721,7 +656,6 @@
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -731,7 +665,6 @@
           <rPr>
             <b/>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -741,7 +674,6 @@
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -751,7 +683,6 @@
           <rPr>
             <b/>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -761,7 +692,6 @@
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -773,20 +703,19 @@
 </comments>
 </file>
 
-<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<file path=xl/comments4.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>Gary Goldstein</author>
     <author>Amit Kanudia</author>
     <author>Maurizio Gargiulo</author>
   </authors>
   <commentList>
-    <comment ref="T3" authorId="0" shapeId="0">
+    <comment ref="T3" authorId="0">
       <text>
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -798,7 +727,6 @@
           <rPr>
             <b/>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -807,7 +735,6 @@
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -818,7 +745,6 @@
           <rPr>
             <b/>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -827,7 +753,6 @@
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -838,7 +763,6 @@
           <rPr>
             <b/>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -847,7 +771,6 @@
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -858,7 +781,6 @@
           <rPr>
             <b/>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -867,7 +789,6 @@
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -878,7 +799,6 @@
           <rPr>
             <b/>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -887,7 +807,6 @@
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -895,13 +814,12 @@
         </r>
       </text>
     </comment>
-    <comment ref="Y3" authorId="1" shapeId="0">
+    <comment ref="Y3" authorId="1">
       <text>
         <r>
           <rPr>
             <b/>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -910,7 +828,6 @@
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -921,12 +838,11 @@
         </r>
       </text>
     </comment>
-    <comment ref="Z3" authorId="2" shapeId="0">
+    <comment ref="Z3" authorId="2">
       <text>
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -936,7 +852,6 @@
           <rPr>
             <b/>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -946,7 +861,6 @@
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -956,7 +870,6 @@
           <rPr>
             <b/>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -966,7 +879,6 @@
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -976,7 +888,6 @@
           <rPr>
             <b/>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -986,7 +897,6 @@
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -994,12 +904,11 @@
         </r>
       </text>
     </comment>
-    <comment ref="AA3" authorId="2" shapeId="0">
+    <comment ref="AA3" authorId="2">
       <text>
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -1009,7 +918,6 @@
           <rPr>
             <b/>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -1019,7 +927,6 @@
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -1029,7 +936,6 @@
           <rPr>
             <b/>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -1039,7 +945,6 @@
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -1047,12 +952,11 @@
         </r>
       </text>
     </comment>
-    <comment ref="AB3" authorId="2" shapeId="0">
+    <comment ref="AB3" authorId="2">
       <text>
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -1063,7 +967,6 @@
           <rPr>
             <b/>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -1072,7 +975,6 @@
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -1080,12 +982,11 @@
         </r>
       </text>
     </comment>
-    <comment ref="Z9" authorId="2" shapeId="0">
+    <comment ref="Z9" authorId="2">
       <text>
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -1096,7 +997,6 @@
           <rPr>
             <b/>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -1105,7 +1005,6 @@
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -1116,7 +1015,6 @@
           <rPr>
             <b/>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -1125,7 +1023,6 @@
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -1136,7 +1033,6 @@
           <rPr>
             <b/>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -1145,7 +1041,6 @@
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -1156,7 +1051,6 @@
           <rPr>
             <b/>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -1165,7 +1059,6 @@
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -1173,13 +1066,12 @@
         </r>
       </text>
     </comment>
-    <comment ref="AA9" authorId="1" shapeId="0">
+    <comment ref="AA9" authorId="1">
       <text>
         <r>
           <rPr>
             <b/>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -1188,7 +1080,6 @@
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -1198,12 +1089,11 @@
         </r>
       </text>
     </comment>
-    <comment ref="AB9" authorId="2" shapeId="0">
+    <comment ref="AB9" authorId="2">
       <text>
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -1213,7 +1103,6 @@
           <rPr>
             <b/>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -1223,7 +1112,6 @@
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -1233,7 +1121,6 @@
           <rPr>
             <b/>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -1242,7 +1129,6 @@
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -1252,7 +1138,6 @@
           <rPr>
             <b/>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -1261,12 +1146,11 @@
         </r>
       </text>
     </comment>
-    <comment ref="T10" authorId="2" shapeId="0">
+    <comment ref="T10" authorId="2">
       <text>
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -1275,7 +1159,6 @@
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -1286,7 +1169,6 @@
           <rPr>
             <b/>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -1296,7 +1178,6 @@
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -1306,7 +1187,6 @@
           <rPr>
             <b/>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -1316,7 +1196,6 @@
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -1326,7 +1205,6 @@
           <rPr>
             <b/>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -1336,7 +1214,6 @@
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -1346,7 +1223,6 @@
           <rPr>
             <b/>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -1356,7 +1232,6 @@
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -1366,7 +1241,6 @@
           <rPr>
             <b/>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -1376,7 +1250,6 @@
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -1386,7 +1259,6 @@
           <rPr>
             <b/>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -1396,7 +1268,6 @@
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -1406,7 +1277,6 @@
           <rPr>
             <b/>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -1416,7 +1286,6 @@
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -1427,7 +1296,6 @@
           <rPr>
             <b/>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -1436,7 +1304,6 @@
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -1446,7 +1313,6 @@
           <rPr>
             <b/>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -1456,7 +1322,6 @@
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -1466,7 +1331,6 @@
           <rPr>
             <b/>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -1476,7 +1340,6 @@
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -1486,7 +1349,6 @@
           <rPr>
             <b/>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -1496,7 +1358,6 @@
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -2027,14 +1888,17 @@
     <numFmt numFmtId="190" formatCode="0.0000"/>
     <numFmt numFmtId="195" formatCode="\Te\x\t"/>
   </numFmts>
-  <fonts count="34" x14ac:knownFonts="1">
+  <fonts count="26">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
+      <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
@@ -2048,11 +1912,6 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
       <b/>
       <sz val="10"/>
       <color indexed="12"/>
@@ -2061,40 +1920,12 @@
     </font>
     <font>
       <sz val="8"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="8"/>
-      <color indexed="81"/>
       <name val="Tahoma"/>
       <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="8"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="8"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="8"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="8"/>
-      <color indexed="81"/>
       <name val="Tahoma"/>
       <family val="2"/>
     </font>
@@ -2116,19 +1947,10 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
       <b/>
       <sz val="14"/>
       <name val="Arial"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
     </font>
     <font>
       <sz val="11"/>
@@ -2209,12 +2031,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
       <b/>
       <sz val="8"/>
       <color theme="1"/>
@@ -2224,7 +2040,7 @@
     <font>
       <b/>
       <sz val="10"/>
-      <color theme="9" tint="-0.249977111117893"/>
+      <color theme="9" tint="-0.249970003962517"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -2252,7 +2068,61 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799979984760284"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599990010261536"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799979984760284"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor indexed="43"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599990010261536"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -2264,80 +2134,31 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.79998168889431442"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.59999389629810485"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.79998168889431442"/>
+        <fgColor theme="4" tint="0.799979984760284"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.59999389629810485"/>
+        <fgColor theme="6" tint="0.799979984760284"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.79998168889431442"/>
+        <fgColor theme="7" tint="0.799979984760284"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.79998168889431442"/>
+        <fgColor theme="3" tint="0.799979984760284"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="3" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.59999389629810485"/>
+        <fgColor theme="9" tint="0.599990010261536"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -2346,173 +2167,6 @@
     <border>
       <left/>
       <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
       <top/>
       <bottom/>
       <diagonal/>
@@ -2530,7 +2184,64 @@
       <bottom style="thin">
         <color rgb="FF7F7F7F"/>
       </bottom>
-      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
     </border>
     <border>
       <left style="thin">
@@ -2540,27 +2251,25 @@
         <color rgb="FF7F7F7F"/>
       </right>
       <top style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </top>
       <bottom style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </bottom>
-      <diagonal/>
     </border>
     <border>
       <left style="thin">
         <color rgb="FF7F7F7F"/>
       </left>
       <right style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </right>
       <top style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </top>
       <bottom style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </bottom>
-      <diagonal/>
     </border>
     <border>
       <left/>
@@ -2568,260 +2277,456 @@
         <color rgb="FF7F7F7F"/>
       </right>
       <top style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </top>
       <bottom style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </bottom>
-      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
     </border>
   </borders>
-  <cellStyleXfs count="30">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="20" fillId="7" borderId="16" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="171" fontId="18" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="21" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="22" fillId="9" borderId="16" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="23" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="15" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="15" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="17" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+  <cellStyleXfs count="48">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
+      <alignment/>
+      <protection/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="171" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
+      <alignment/>
+      <protection/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
+      <alignment/>
+      <protection/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
+      <alignment/>
+      <protection/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
+      <alignment/>
+      <protection/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0">
+      <alignment/>
+      <protection/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
+      <alignment/>
+      <protection/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0">
+      <alignment/>
+      <protection/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
+      <alignment/>
+      <protection/>
+    </xf>
   </cellStyleXfs>
   <cellXfs count="122">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="11" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="30" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="11" applyFont="1" applyFill="1" applyAlignment="1">
+      <protection/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="30" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="11" applyFill="1" applyBorder="1" applyAlignment="1">
+      <protection/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="30" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
+      <protection/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment/>
+    </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="0" xfId="3"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="6" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="24" fillId="11" borderId="0" xfId="6" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="8" applyFont="1" applyFill="1"/>
-    <xf numFmtId="1" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="25" fillId="4" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="0" xfId="22"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="25" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" xfId="25" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="27" applyFont="1" applyFill="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="3" xfId="20" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="4" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="3" xfId="20" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="4" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="4" xfId="20" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="11" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="4" xfId="30" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="11" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <protection/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="4" xfId="30" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="11" borderId="0" xfId="6" applyFont="1" applyFill="1" applyAlignment="1">
+      <protection/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" xfId="25" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="0" xfId="3" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="0" xfId="22" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="9"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="9" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="9" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="9" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="9" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="28">
+      <alignment/>
+      <protection/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="28" applyFill="1">
+      <alignment/>
+      <protection/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="28" applyFill="1" applyBorder="1">
+      <alignment/>
+      <protection/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="28" applyBorder="1">
+      <alignment/>
+      <protection/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="28" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="11" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <protection/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="30" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
+      <protection/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="6" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="25" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="22" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="29" fillId="12" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="1" fillId="11" borderId="0" xfId="21" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="21" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="21" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="29" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="21" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="5" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="5" xfId="21" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="3" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="22" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="11" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="9" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
+      <alignment/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
+      <alignment/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="30" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="11" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <protection/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="3" xfId="30" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="24" fillId="11" borderId="0" xfId="6" applyFont="1" applyFill="1" applyAlignment="1">
+      <protection/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" xfId="25" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="1" fontId="0" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="23" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="1" fontId="0" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="1" fontId="22" fillId="9" borderId="0" xfId="7" applyNumberFormat="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="1" fontId="22" fillId="9" borderId="5" xfId="7" applyNumberFormat="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="187" fontId="20" fillId="7" borderId="6" xfId="4" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="15" fillId="7" borderId="0" xfId="26" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment/>
+    </xf>
+    <xf numFmtId="1" fontId="15" fillId="7" borderId="6" xfId="26" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment/>
+    </xf>
+    <xf numFmtId="187" fontId="13" fillId="5" borderId="7" xfId="23" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="20" fillId="7" borderId="17" xfId="4" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="13" fillId="5" borderId="8" xfId="23" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="1" fontId="20" fillId="7" borderId="18" xfId="4" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="13" fillId="5" borderId="9" xfId="23" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="1" fontId="20" fillId="7" borderId="19" xfId="4" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="13" fillId="5" borderId="10" xfId="23" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="187" fontId="13" fillId="14" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="187" fontId="8" fillId="14" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="187" fontId="13" fillId="14" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="187" fontId="8" fillId="14" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="13" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="13" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="187" fontId="13" fillId="15" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="187" fontId="8" fillId="15" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="13" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="13" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="13" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="13" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="13" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="13" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="6" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="4" borderId="2" xfId="22" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="188" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="9" fontId="4" fillId="16" borderId="0" xfId="16" applyFont="1" applyFill="1"/>
-    <xf numFmtId="2" fontId="4" fillId="14" borderId="0" xfId="8" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="14" borderId="0" xfId="8" applyFont="1" applyFill="1"/>
+    <xf numFmtId="9" fontId="0" fillId="16" borderId="0" xfId="15" applyFont="1" applyFill="1"/>
+    <xf numFmtId="2" fontId="0" fillId="14" borderId="0" xfId="27" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="27" applyFont="1" applyFill="1"/>
     <xf numFmtId="2" fontId="0" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="14" borderId="0" xfId="9" applyFill="1"/>
-    <xf numFmtId="2" fontId="4" fillId="14" borderId="0" xfId="9" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="0" xfId="8" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="28" applyFill="1">
+      <alignment/>
+      <protection/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="14" borderId="0" xfId="28" applyNumberFormat="1" applyFill="1">
+      <alignment/>
+      <protection/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="27" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="11" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="4" xfId="30" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="4" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <protection/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="16" xfId="20" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="12" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="4" xfId="31" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="187" fontId="12" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <protection/>
+    </xf>
+    <xf numFmtId="187" fontId="7" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="1" fontId="3" fillId="14" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="25" fillId="4" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="14" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="5" xfId="20" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="20" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="187" fontId="13" fillId="15" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="187" fontId="8" fillId="15" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="187" fontId="13" fillId="15" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="187" fontId="8" fillId="15" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="188" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="14" borderId="0" xfId="9" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="4" fillId="14" borderId="0" xfId="9" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="22" fillId="0" borderId="0" xfId="7" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="28" applyFill="1" applyBorder="1">
+      <alignment/>
+      <protection/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="14" borderId="0" xfId="28" applyNumberFormat="1" applyFill="1" applyBorder="1">
+      <alignment/>
+      <protection/>
+    </xf>
+    <xf numFmtId="1" fontId="15" fillId="0" borderId="0" xfId="26" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment/>
+    </xf>
     <xf numFmtId="186" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="1" fontId="4" fillId="0" borderId="0" xfId="9" applyNumberFormat="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="28" applyNumberFormat="1">
+      <alignment/>
+      <protection/>
+    </xf>
     <xf numFmtId="1" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="1" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="25" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="18" fillId="0" borderId="0" xfId="21" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="5" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="3" borderId="5" xfId="21" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="12" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="11" borderId="3" xfId="21" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="190" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="188" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="25" fillId="4" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="3" xfId="20" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="195" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="195" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="195" fontId="3" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="195" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="195" fontId="3" fillId="10" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="195" fontId="3" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="195" fontId="3" fillId="10" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="195" fontId="25" fillId="4" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="195" fontId="18" fillId="2" borderId="3" xfId="20" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="195" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
@@ -2829,57 +2734,133 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="195" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="195" fontId="25" fillId="4" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="195" fontId="18" fillId="2" borderId="3" xfId="20" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="195" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="195" fontId="4" fillId="0" borderId="0" xfId="9" applyNumberFormat="1"/>
+    <xf numFmtId="195" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="195" fontId="0" fillId="0" borderId="0" xfId="28" applyNumberFormat="1">
+      <alignment/>
+      <protection/>
+    </xf>
     <xf numFmtId="195" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="195" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="195" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="30">
-    <cellStyle name="20% - Accent5" xfId="1" builtinId="46"/>
-    <cellStyle name="40% - Accent3" xfId="2" builtinId="39"/>
-    <cellStyle name="Accent2" xfId="3" builtinId="33"/>
-    <cellStyle name="Calculation" xfId="4" builtinId="22"/>
-    <cellStyle name="Comma 2" xfId="5"/>
-    <cellStyle name="Good" xfId="6" builtinId="26"/>
-    <cellStyle name="Input" xfId="7" builtinId="20"/>
-    <cellStyle name="Neutral" xfId="8" builtinId="28"/>
+  <cellStyles count="34">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 10" xfId="9"/>
-    <cellStyle name="Normal 2" xfId="10"/>
-    <cellStyle name="Normal 4" xfId="11"/>
-    <cellStyle name="Normal 4 2" xfId="12"/>
-    <cellStyle name="Normal 8" xfId="13"/>
-    <cellStyle name="Normal 9 2" xfId="14"/>
-    <cellStyle name="Normale_B2020" xfId="15"/>
-    <cellStyle name="Percent" xfId="16" builtinId="5"/>
-    <cellStyle name="Percent 2" xfId="17"/>
-    <cellStyle name="Percent 3" xfId="18"/>
-    <cellStyle name="Percent 3 2" xfId="19"/>
-    <cellStyle name="Percent 3 3" xfId="20"/>
-    <cellStyle name="Percent 3 4" xfId="21"/>
-    <cellStyle name="Percent 4" xfId="22"/>
-    <cellStyle name="Percent 4 2" xfId="23"/>
-    <cellStyle name="Percent 4 3" xfId="24"/>
-    <cellStyle name="Percent 4 4" xfId="25"/>
-    <cellStyle name="Percent 5" xfId="26"/>
-    <cellStyle name="Percent 6" xfId="27"/>
-    <cellStyle name="Percent 7" xfId="28"/>
-    <cellStyle name="Standard_Sce_D_Extraction" xfId="29"/>
+    <cellStyle name="Percent" xfId="15" builtinId="5"/>
+    <cellStyle name="Currency" xfId="16" builtinId="4"/>
+    <cellStyle name="Currency [0]" xfId="17" builtinId="7"/>
+    <cellStyle name="Comma" xfId="18" builtinId="3"/>
+    <cellStyle name="Comma [0]" xfId="19" builtinId="6"/>
+    <cellStyle name="20% - Accent5" xfId="20" builtinId="46"/>
+    <cellStyle name="40% - Accent3" xfId="21" builtinId="39"/>
+    <cellStyle name="Accent2" xfId="22" builtinId="33"/>
+    <cellStyle name="Calculation" xfId="23" builtinId="22"/>
+    <cellStyle name="Comma 2" xfId="24"/>
+    <cellStyle name="Good" xfId="25" builtinId="26"/>
+    <cellStyle name="Input" xfId="26" builtinId="20"/>
+    <cellStyle name="Neutral" xfId="27" builtinId="28"/>
+    <cellStyle name="Normal 10" xfId="28"/>
+    <cellStyle name="Normal 2" xfId="29"/>
+    <cellStyle name="Normal 4" xfId="30"/>
+    <cellStyle name="Normal 4 2" xfId="31"/>
+    <cellStyle name="Normal 8" xfId="32"/>
+    <cellStyle name="Normal 9 2" xfId="33"/>
+    <cellStyle name="Normale_B2020" xfId="34"/>
+    <cellStyle name="Percent 2" xfId="35"/>
+    <cellStyle name="Percent 3" xfId="36"/>
+    <cellStyle name="Percent 3 2" xfId="37"/>
+    <cellStyle name="Percent 3 3" xfId="38"/>
+    <cellStyle name="Percent 3 4" xfId="39"/>
+    <cellStyle name="Percent 4" xfId="40"/>
+    <cellStyle name="Percent 4 2" xfId="41"/>
+    <cellStyle name="Percent 4 3" xfId="42"/>
+    <cellStyle name="Percent 4 4" xfId="43"/>
+    <cellStyle name="Percent 5" xfId="44"/>
+    <cellStyle name="Percent 6" xfId="45"/>
+    <cellStyle name="Percent 7" xfId="46"/>
+    <cellStyle name="Standard_Sce_D_Extraction" xfId="47"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -2892,7 +2873,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
@@ -2911,7 +2892,7 @@
         <xdr:cNvPr id="56975" name="Picture 6">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{07B54768-2264-459D-AAAF-4E7CAD4688C6}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{07b54768-2264-459d-aaaf-4e7cad4688c6}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2920,14 +2901,13 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+        <a:blip r:embed="rId1">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main"/>
             </a:ext>
           </a:extLst>
         </a:blip>
-        <a:srcRect/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -2937,9 +2917,7 @@
           <a:off x="123825" y="962025"/>
           <a:ext cx="800100" cy="2238375"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
+        <a:prstGeom prst="rect"/>
         <a:noFill/>
         <a:ln>
           <a:noFill/>
@@ -2985,7 +2963,7 @@
         <xdr:cNvPr id="56976" name="Picture 8">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{092998F4-DAF5-4AB5-A34B-DFA9CC7FF7F7}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{092998f4-daf5-4ab5-a34b-dfa9cc7ff7f7}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2994,14 +2972,13 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
+        <a:blip r:embed="rId2">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main"/>
             </a:ext>
           </a:extLst>
         </a:blip>
-        <a:srcRect/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -3011,9 +2988,7 @@
           <a:off x="1552575" y="18926175"/>
           <a:ext cx="4019550" cy="1905000"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
+        <a:prstGeom prst="rect"/>
         <a:noFill/>
         <a:ln>
           <a:noFill/>
@@ -3059,7 +3034,7 @@
         <xdr:cNvPr id="56977" name="Picture 4">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AD288841-D70D-4C2E-9A6A-06C46B032C2B}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{ad288841-d70d-4c2e-9a6a-06c46b032c2b}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3068,14 +3043,13 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3">
+        <a:blip r:embed="rId3">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main"/>
             </a:ext>
           </a:extLst>
         </a:blip>
-        <a:srcRect/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -3085,9 +3059,7 @@
           <a:off x="1552575" y="1104900"/>
           <a:ext cx="6524625" cy="3905250"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
+        <a:prstGeom prst="rect"/>
         <a:noFill/>
         <a:ln>
           <a:noFill/>
@@ -3133,7 +3105,7 @@
         <xdr:cNvPr id="56978" name="Picture 5">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F7EDBE9C-2FFC-4928-AE9B-DF9BBBDE5C06}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{f7edbe9c-2ffc-4928-ae9b-df9bbbde5c06}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3142,14 +3114,13 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4">
+        <a:blip r:embed="rId4">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main"/>
             </a:ext>
           </a:extLst>
         </a:blip>
-        <a:srcRect/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -3159,9 +3130,7 @@
           <a:off x="1552575" y="4962525"/>
           <a:ext cx="3343275" cy="952500"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
+        <a:prstGeom prst="rect"/>
         <a:noFill/>
         <a:ln>
           <a:noFill/>
@@ -3193,7 +3162,7 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>10</xdr:col>
@@ -3207,12 +3176,12 @@
       <xdr:row>33</xdr:row>
       <xdr:rowOff>19049</xdr:rowOff>
     </xdr:to>
-    <xdr:sp macro="" textlink="">
+    <xdr:sp>
       <xdr:nvSpPr>
         <xdr:cNvPr id="2" name="TextBox 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F6B2F145-8850-4388-9ADE-B2C38CEC5F7B}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{f6b2f145-8850-4388-9ade-b2c38cec5f7b}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3220,12 +3189,10 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="6537960" y="4933949"/>
-          <a:ext cx="6376035" cy="981075"/>
+          <a:off x="6534150" y="4933950"/>
+          <a:ext cx="6372225" cy="981075"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
+        <a:prstGeom prst="rect"/>
         <a:solidFill>
           <a:schemeClr val="accent6">
             <a:lumMod val="20000"/>
@@ -3234,7 +3201,7 @@
         </a:solidFill>
         <a:ln w="9525" cmpd="sng">
           <a:solidFill>
-            <a:schemeClr val="lt1">
+            <a:schemeClr val="bg1">
               <a:shade val="50000"/>
             </a:schemeClr>
           </a:solidFill>
@@ -3242,16 +3209,16 @@
       </xdr:spPr>
       <xdr:style>
         <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
+          <a:srgbClr val="000000"/>
         </a:lnRef>
         <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
+          <a:srgbClr val="000000"/>
         </a:fillRef>
         <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
+          <a:srgbClr val="000000"/>
         </a:effectRef>
         <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
+          <a:schemeClr val="tx1"/>
         </a:fontRef>
       </xdr:style>
       <xdr:txBody>
@@ -3262,7 +3229,7 @@
           <a:r>
             <a:rPr lang="en-GB" sz="1100">
               <a:solidFill>
-                <a:schemeClr val="dk1"/>
+                <a:schemeClr val="tx1"/>
               </a:solidFill>
               <a:effectLst/>
               <a:latin typeface="+mn-lt"/>
@@ -3274,7 +3241,7 @@
           <a:r>
             <a:rPr lang="en-GB" sz="1100" baseline="0">
               <a:solidFill>
-                <a:schemeClr val="dk1"/>
+                <a:schemeClr val="tx1"/>
               </a:solidFill>
               <a:effectLst/>
               <a:latin typeface="+mn-lt"/>
@@ -3286,7 +3253,7 @@
           <a:r>
             <a:rPr lang="en-GB" sz="1100">
               <a:solidFill>
-                <a:schemeClr val="dk1"/>
+                <a:schemeClr val="tx1"/>
               </a:solidFill>
               <a:effectLst/>
               <a:latin typeface="+mn-lt"/>
@@ -3300,7 +3267,7 @@
           <a:pPr lvl="0"/>
           <a:endParaRPr lang="en-GB" sz="1100">
             <a:solidFill>
-              <a:schemeClr val="dk1"/>
+              <a:schemeClr val="tx1"/>
             </a:solidFill>
             <a:effectLst/>
             <a:latin typeface="+mn-lt"/>
@@ -3313,7 +3280,7 @@
           <a:r>
             <a:rPr lang="en-GB" sz="1100">
               <a:solidFill>
-                <a:schemeClr val="dk1"/>
+                <a:schemeClr val="tx1"/>
               </a:solidFill>
               <a:effectLst/>
               <a:latin typeface="+mn-lt"/>
@@ -3325,7 +3292,7 @@
           <a:r>
             <a:rPr lang="en-GB" sz="1100" baseline="0">
               <a:solidFill>
-                <a:schemeClr val="dk1"/>
+                <a:schemeClr val="tx1"/>
               </a:solidFill>
               <a:effectLst/>
               <a:latin typeface="+mn-lt"/>
@@ -3336,7 +3303,7 @@
           </a:r>
           <a:endParaRPr lang="en-GB" sz="1100">
             <a:solidFill>
-              <a:schemeClr val="dk1"/>
+              <a:schemeClr val="tx1"/>
             </a:solidFill>
             <a:effectLst/>
             <a:latin typeface="+mn-lt"/>
@@ -3352,7 +3319,7 @@
 </file>
 
 <file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>19</xdr:col>
@@ -3366,12 +3333,12 @@
       <xdr:row>29</xdr:row>
       <xdr:rowOff>1090</xdr:rowOff>
     </xdr:to>
-    <xdr:sp macro="" textlink="">
+    <xdr:sp>
       <xdr:nvSpPr>
         <xdr:cNvPr id="2" name="TextBox 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{32D1CAE3-AB1F-44E7-83A8-8CFE9F3A6676}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{32d1cae3-ab1f-44e7-83a8-8cfe9f3a6676}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3379,12 +3346,10 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="10692974" y="4231428"/>
-          <a:ext cx="6483756" cy="1262412"/>
+          <a:off x="12925425" y="4276725"/>
+          <a:ext cx="6477000" cy="1285875"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
+        <a:prstGeom prst="rect"/>
         <a:solidFill>
           <a:schemeClr val="accent6">
             <a:lumMod val="20000"/>
@@ -3393,7 +3358,7 @@
         </a:solidFill>
         <a:ln w="9525" cmpd="sng">
           <a:solidFill>
-            <a:schemeClr val="lt1">
+            <a:schemeClr val="bg1">
               <a:shade val="50000"/>
             </a:schemeClr>
           </a:solidFill>
@@ -3401,16 +3366,16 @@
       </xdr:spPr>
       <xdr:style>
         <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
+          <a:srgbClr val="000000"/>
         </a:lnRef>
         <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
+          <a:srgbClr val="000000"/>
         </a:fillRef>
         <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
+          <a:srgbClr val="000000"/>
         </a:effectRef>
         <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
+          <a:schemeClr val="tx1"/>
         </a:fontRef>
       </xdr:style>
       <xdr:txBody>
@@ -3421,7 +3386,7 @@
           <a:r>
             <a:rPr lang="en-GB" sz="1100">
               <a:solidFill>
-                <a:schemeClr val="dk1"/>
+                <a:schemeClr val="tx1"/>
               </a:solidFill>
               <a:effectLst/>
               <a:latin typeface="+mn-lt"/>
@@ -3433,7 +3398,7 @@
           <a:r>
             <a:rPr lang="en-GB" sz="1100" baseline="0">
               <a:solidFill>
-                <a:schemeClr val="dk1"/>
+                <a:schemeClr val="tx1"/>
               </a:solidFill>
               <a:effectLst/>
               <a:latin typeface="+mn-lt"/>
@@ -3445,7 +3410,7 @@
           <a:r>
             <a:rPr lang="en-GB" sz="1100">
               <a:solidFill>
-                <a:schemeClr val="dk1"/>
+                <a:schemeClr val="tx1"/>
               </a:solidFill>
               <a:effectLst/>
               <a:latin typeface="+mn-lt"/>
@@ -3459,7 +3424,7 @@
           <a:pPr lvl="0"/>
           <a:endParaRPr lang="en-GB" sz="1100">
             <a:solidFill>
-              <a:schemeClr val="dk1"/>
+              <a:schemeClr val="tx1"/>
             </a:solidFill>
             <a:effectLst/>
             <a:latin typeface="+mn-lt"/>
@@ -3472,7 +3437,7 @@
           <a:r>
             <a:rPr lang="en-GB" sz="1100">
               <a:solidFill>
-                <a:schemeClr val="dk1"/>
+                <a:schemeClr val="tx1"/>
               </a:solidFill>
               <a:effectLst/>
               <a:latin typeface="+mn-lt"/>
@@ -3490,7 +3455,7 @@
 </file>
 
 <file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>1</xdr:col>
@@ -3504,12 +3469,12 @@
       <xdr:row>15</xdr:row>
       <xdr:rowOff>66675</xdr:rowOff>
     </xdr:to>
-    <xdr:sp macro="" textlink="">
+    <xdr:sp>
       <xdr:nvSpPr>
         <xdr:cNvPr id="2" name="TextBox 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BD1A3727-B21E-4010-995E-8645C474E6C5}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{bd1a3727-b21e-4010-995e-8645c474e6c5}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3517,12 +3482,10 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="609600" y="1971675"/>
+          <a:off x="609600" y="2143125"/>
           <a:ext cx="4391025" cy="552450"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
+        <a:prstGeom prst="rect"/>
         <a:solidFill>
           <a:schemeClr val="accent6">
             <a:lumMod val="20000"/>
@@ -3531,7 +3494,7 @@
         </a:solidFill>
         <a:ln w="9525" cmpd="sng">
           <a:solidFill>
-            <a:schemeClr val="lt1">
+            <a:schemeClr val="bg1">
               <a:shade val="50000"/>
             </a:schemeClr>
           </a:solidFill>
@@ -3539,16 +3502,16 @@
       </xdr:spPr>
       <xdr:style>
         <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
+          <a:srgbClr val="000000"/>
         </a:lnRef>
         <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
+          <a:srgbClr val="000000"/>
         </a:fillRef>
         <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
+          <a:srgbClr val="000000"/>
         </a:effectRef>
         <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
+          <a:schemeClr val="tx1"/>
         </a:fontRef>
       </xdr:style>
       <xdr:txBody>
@@ -3559,7 +3522,7 @@
           <a:r>
             <a:rPr lang="en-GB" sz="1100">
               <a:solidFill>
-                <a:schemeClr val="dk1"/>
+                <a:schemeClr val="tx1"/>
               </a:solidFill>
               <a:effectLst/>
               <a:latin typeface="+mn-lt"/>
@@ -3571,7 +3534,7 @@
           <a:r>
             <a:rPr lang="en-GB" sz="1100" baseline="0">
               <a:solidFill>
-                <a:schemeClr val="dk1"/>
+                <a:schemeClr val="tx1"/>
               </a:solidFill>
               <a:effectLst/>
               <a:latin typeface="+mn-lt"/>
@@ -3582,7 +3545,7 @@
           </a:r>
           <a:endParaRPr lang="en-GB" sz="1100">
             <a:solidFill>
-              <a:schemeClr val="dk1"/>
+              <a:schemeClr val="tx1"/>
             </a:solidFill>
             <a:effectLst/>
             <a:latin typeface="+mn-lt"/>
@@ -3598,7 +3561,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="IEA Data"/>
@@ -3733,7 +3696,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="EnergyBalance"/>
@@ -3746,28 +3709,28 @@
       <sheetData sheetId="1">
         <row r="10">
           <cell r="D10">
-            <v>-37.464700000000001</v>
+            <v>-37.4647</v>
           </cell>
           <cell r="E10">
-            <v>-317.19200000000001</v>
+            <v>-317.192</v>
           </cell>
           <cell r="F10">
             <v>0</v>
           </cell>
           <cell r="G10">
-            <v>-16.283999999999999</v>
+            <v>-16.284</v>
           </cell>
           <cell r="H10">
-            <v>-2.1499999999999998E-2</v>
+            <v>-0.0215</v>
           </cell>
           <cell r="I10">
-            <v>-528.76099999999997</v>
+            <v>-528.761</v>
           </cell>
           <cell r="J10">
-            <v>-164.50800000000001</v>
+            <v>-164.508</v>
           </cell>
           <cell r="K10">
-            <v>-0.61599999999999999</v>
+            <v>-0.616</v>
           </cell>
           <cell r="L10">
             <v>-205.88</v>
@@ -3800,27 +3763,27 @@
             <v>0</v>
           </cell>
           <cell r="V10">
-            <v>-1274.6994499999998</v>
+            <v>-1274.69945</v>
           </cell>
         </row>
         <row r="11">
           <cell r="D11">
-            <v>-6238.7780000000012</v>
+            <v>-6238.778</v>
           </cell>
           <cell r="E11">
-            <v>-2254.2175999999999</v>
+            <v>-2254.2176</v>
           </cell>
           <cell r="F11">
             <v>0</v>
           </cell>
           <cell r="G11">
-            <v>-30.160499999999999</v>
+            <v>-30.1605</v>
           </cell>
           <cell r="H11">
             <v>0</v>
           </cell>
           <cell r="I11">
-            <v>-23.835000000000001</v>
+            <v>-23.835</v>
           </cell>
           <cell r="J11">
             <v>0</v>
@@ -3832,16 +3795,16 @@
             <v>-524.78</v>
           </cell>
           <cell r="M11">
-            <v>-33.529000000000003</v>
+            <v>-33.529</v>
           </cell>
           <cell r="N11">
             <v>-4455</v>
           </cell>
           <cell r="O11">
-            <v>-527.25918750000005</v>
+            <v>-527.2591875</v>
           </cell>
           <cell r="P11">
-            <v>-502.66000000000008</v>
+            <v>-502.66</v>
           </cell>
           <cell r="Q11">
             <v>-263.8965</v>
@@ -3850,16 +3813,16 @@
             <v>-68</v>
           </cell>
           <cell r="S11">
-            <v>-16.474499999999999</v>
+            <v>-16.4745</v>
           </cell>
           <cell r="T11">
-            <v>868.77949999999998</v>
+            <v>868.7795</v>
           </cell>
           <cell r="U11">
             <v>5790.5</v>
           </cell>
           <cell r="V11">
-            <v>-8279.3107875000023</v>
+            <v>-8279.3107875</v>
           </cell>
         </row>
         <row r="12">
@@ -3873,13 +3836,13 @@
             <v>0</v>
           </cell>
           <cell r="G12">
-            <v>-7.6189999999999998</v>
+            <v>-7.619</v>
           </cell>
           <cell r="H12">
             <v>0</v>
           </cell>
           <cell r="I12">
-            <v>-0.23350000000000001</v>
+            <v>-0.2335</v>
           </cell>
           <cell r="J12">
             <v>0</v>
@@ -3909,16 +3872,16 @@
             <v>0</v>
           </cell>
           <cell r="S12">
-            <v>-0.78449999999999998</v>
+            <v>-0.7845</v>
           </cell>
           <cell r="T12">
-            <v>329.37150000000003</v>
+            <v>329.3715</v>
           </cell>
           <cell r="U12">
             <v>0</v>
           </cell>
           <cell r="V12">
-            <v>-26.820549999999912</v>
+            <v>-26.8205499999999</v>
           </cell>
         </row>
         <row r="13">
@@ -3935,22 +3898,22 @@
             <v>5701.34</v>
           </cell>
           <cell r="H13">
-            <v>969.47799999999995</v>
+            <v>969.478</v>
           </cell>
           <cell r="I13">
-            <v>1086.3040000000001</v>
+            <v>1086.304</v>
           </cell>
           <cell r="J13">
-            <v>3354.9119999999998</v>
+            <v>3354.912</v>
           </cell>
           <cell r="K13">
-            <v>970.28800000000001</v>
+            <v>970.288</v>
           </cell>
           <cell r="L13">
-            <v>2285.1019999999999</v>
+            <v>2285.102</v>
           </cell>
           <cell r="M13">
-            <v>1299.9449999999999</v>
+            <v>1299.945</v>
           </cell>
           <cell r="N13">
             <v>0</v>
@@ -3977,7 +3940,7 @@
             <v>0</v>
           </cell>
           <cell r="V13">
-            <v>-200.86150000000021</v>
+            <v>-200.8615</v>
           </cell>
         </row>
       </sheetData>
@@ -4335,29 +4298,29 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
-    <tabColor theme="5" tint="-0.249977111117893"/>
+    <tabColor theme="5" tint="-0.249970003962517"/>
   </sheetPr>
   <dimension ref="A1:AA17"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" width="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="41.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="7" width="10.85546875" customWidth="1"/>
-    <col min="8" max="8" width="12.140625" customWidth="1"/>
-    <col min="9" max="12" width="10.85546875" customWidth="1"/>
-    <col min="13" max="13" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="14" max="21" width="10.85546875" customWidth="1"/>
-    <col min="22" max="22" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.5714285714286" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="41.1428571428571" bestFit="1" customWidth="1"/>
+    <col min="4" max="7" width="10.8571428571429" customWidth="1"/>
+    <col min="8" max="8" width="12.1428571428571" customWidth="1"/>
+    <col min="9" max="12" width="10.8571428571429" customWidth="1"/>
+    <col min="13" max="13" width="17.8571428571429" bestFit="1" customWidth="1"/>
+    <col min="14" max="21" width="10.8571428571429" customWidth="1"/>
+    <col min="22" max="22" width="7.28571428571429" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="2" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="6.7109375" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="12.5714285714286" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="6.71428571428571" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="9.28571428571429" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" s="6" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="24:27" s="6" customFormat="1" ht="12.75">
       <c r="X1" s="23" t="s">
         <v>78</v>
       </c>
@@ -4371,7 +4334,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="2" spans="1:27" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="3:27" ht="15.75">
       <c r="C2" s="7"/>
       <c r="D2" s="48" t="s">
         <v>42</v>
@@ -4441,7 +4404,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="3" spans="1:27" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="3" spans="3:22" ht="25.5">
       <c r="C3" s="67" t="s">
         <v>121</v>
       </c>
@@ -4503,7 +4466,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="4" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="4" spans="2:24" ht="12.75">
       <c r="B4" s="46"/>
       <c r="C4" s="83" t="s">
         <v>55</v>
@@ -4529,7 +4492,7 @@
       <c r="V4" s="84"/>
       <c r="X4" s="6"/>
     </row>
-    <row r="5" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:24" ht="12.75">
       <c r="B5" s="50" t="s">
         <v>56</v>
       </c>
@@ -4537,84 +4500,84 @@
         <v>57</v>
       </c>
       <c r="D5" s="51">
-        <f>[2]EB1!D10</f>
+        <f>'[2]EB1'!D10</f>
         <v>-37.464700000000001</v>
       </c>
       <c r="E5" s="51">
-        <f>[2]EB1!E10</f>
+        <f>'[2]EB1'!E10</f>
         <v>-317.19200000000001</v>
       </c>
       <c r="F5" s="51">
-        <f>[2]EB1!F10</f>
+        <f>'[2]EB1'!F10</f>
         <v>0</v>
       </c>
       <c r="G5" s="51">
-        <f>[2]EB1!G10</f>
+        <f>'[2]EB1'!G10</f>
         <v>-16.283999999999999</v>
       </c>
       <c r="H5" s="51">
-        <f>[2]EB1!H10</f>
-        <v>-2.1499999999999998E-2</v>
+        <f>'[2]EB1'!H10</f>
+        <v>-0.021499999999999998</v>
       </c>
       <c r="I5" s="51">
-        <f>[2]EB1!I10</f>
+        <f>'[2]EB1'!I10</f>
         <v>-528.76099999999997</v>
       </c>
       <c r="J5" s="51">
-        <f>[2]EB1!J10</f>
+        <f>'[2]EB1'!J10</f>
         <v>-164.50800000000001</v>
       </c>
       <c r="K5" s="51">
-        <f>[2]EB1!K10</f>
+        <f>'[2]EB1'!K10</f>
         <v>-0.61599999999999999</v>
       </c>
       <c r="L5" s="51">
-        <f>[2]EB1!L10</f>
+        <f>'[2]EB1'!L10</f>
         <v>-205.88</v>
       </c>
       <c r="M5" s="51">
-        <f>[2]EB1!M10</f>
+        <f>'[2]EB1'!M10</f>
         <v>0</v>
       </c>
       <c r="N5" s="51">
-        <f>[2]EB1!N10</f>
+        <f>'[2]EB1'!N10</f>
         <v>0</v>
       </c>
       <c r="O5" s="51">
-        <f>[2]EB1!O10</f>
+        <f>'[2]EB1'!O10</f>
         <v>-3.21225</v>
       </c>
       <c r="P5" s="51">
-        <f>[2]EB1!P10</f>
+        <f>'[2]EB1'!P10</f>
         <v>0</v>
       </c>
       <c r="Q5" s="51">
-        <f>[2]EB1!Q10</f>
+        <f>'[2]EB1'!Q10</f>
         <v>0</v>
       </c>
       <c r="R5" s="51">
-        <f>[2]EB1!R10</f>
+        <f>'[2]EB1'!R10</f>
         <v>0</v>
       </c>
       <c r="S5" s="51">
-        <f>[2]EB1!S10</f>
-        <v>-0.76</v>
+        <f>'[2]EB1'!S10</f>
+        <v>-0.76000000000000001</v>
       </c>
       <c r="T5" s="51">
-        <f>[2]EB1!T10</f>
+        <f>'[2]EB1'!T10</f>
         <v>0</v>
       </c>
       <c r="U5" s="51">
-        <f>[2]EB1!U10</f>
+        <f>'[2]EB1'!U10</f>
         <v>0</v>
       </c>
       <c r="V5" s="85">
-        <f>[2]EB1!V10</f>
+        <f>'[2]EB1'!V10</f>
         <v>-1274.6994499999998</v>
       </c>
       <c r="X5" s="6"/>
     </row>
-    <row r="6" spans="1:27" ht="15" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:24" ht="15">
       <c r="B6" s="50" t="s">
         <v>48</v>
       </c>
@@ -4622,84 +4585,84 @@
         <v>58</v>
       </c>
       <c r="D6" s="54">
-        <f>[2]EB1!D11</f>
+        <f>'[2]EB1'!D11</f>
         <v>-6238.7780000000012</v>
       </c>
       <c r="E6" s="53">
-        <f>[2]EB1!E11</f>
+        <f>'[2]EB1'!E11</f>
         <v>-2254.2175999999999</v>
       </c>
       <c r="F6" s="53">
-        <f>[2]EB1!F11</f>
+        <f>'[2]EB1'!F11</f>
         <v>0</v>
       </c>
       <c r="G6" s="53">
-        <f>[2]EB1!G11</f>
+        <f>'[2]EB1'!G11</f>
         <v>-30.160499999999999</v>
       </c>
       <c r="H6" s="53">
-        <f>[2]EB1!H11</f>
+        <f>'[2]EB1'!H11</f>
         <v>0</v>
       </c>
       <c r="I6" s="53">
-        <f>[2]EB1!I11</f>
+        <f>'[2]EB1'!I11</f>
         <v>-23.835000000000001</v>
       </c>
       <c r="J6" s="53">
-        <f>[2]EB1!J11</f>
+        <f>'[2]EB1'!J11</f>
         <v>0</v>
       </c>
       <c r="K6" s="53">
-        <f>[2]EB1!K11</f>
+        <f>'[2]EB1'!K11</f>
         <v>0</v>
       </c>
       <c r="L6" s="53">
-        <f>[2]EB1!L11</f>
-        <v>-524.78</v>
+        <f>'[2]EB1'!L11</f>
+        <v>-524.77999999999997</v>
       </c>
       <c r="M6" s="53">
-        <f>[2]EB1!M11</f>
+        <f>'[2]EB1'!M11</f>
         <v>-33.529000000000003</v>
       </c>
       <c r="N6" s="53">
-        <f>[2]EB1!N11</f>
+        <f>'[2]EB1'!N11</f>
         <v>-4455</v>
       </c>
       <c r="O6" s="53">
-        <f>[2]EB1!O11</f>
+        <f>'[2]EB1'!O11</f>
         <v>-527.25918750000005</v>
       </c>
       <c r="P6" s="53">
-        <f>[2]EB1!P11</f>
+        <f>'[2]EB1'!P11</f>
         <v>-502.66000000000008</v>
       </c>
       <c r="Q6" s="53">
-        <f>[2]EB1!Q11</f>
+        <f>'[2]EB1'!Q11</f>
         <v>-263.8965</v>
       </c>
       <c r="R6" s="53">
-        <f>[2]EB1!R11</f>
+        <f>'[2]EB1'!R11</f>
         <v>-68</v>
       </c>
       <c r="S6" s="51">
-        <f>[2]EB1!S11</f>
+        <f>'[2]EB1'!S11</f>
         <v>-16.474499999999999</v>
       </c>
       <c r="T6" s="51">
-        <f>[2]EB1!T11</f>
+        <f>'[2]EB1'!T11</f>
         <v>868.77949999999998</v>
       </c>
       <c r="U6" s="53">
-        <f>[2]EB1!U11</f>
+        <f>'[2]EB1'!U11</f>
         <v>5790.5</v>
       </c>
       <c r="V6" s="85">
-        <f>[2]EB1!V11</f>
+        <f>'[2]EB1'!V11</f>
         <v>-8279.3107875000023</v>
       </c>
       <c r="X6" s="95"/>
     </row>
-    <row r="7" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="7" spans="2:24" ht="12.75">
       <c r="B7" s="50" t="s">
         <v>59</v>
       </c>
@@ -4707,84 +4670,84 @@
         <v>60</v>
       </c>
       <c r="D7" s="51">
-        <f>[2]EB1!D12</f>
+        <f>'[2]EB1'!D12</f>
         <v>-104.9074</v>
       </c>
       <c r="E7" s="51">
-        <f>[2]EB1!E12</f>
+        <f>'[2]EB1'!E12</f>
         <v>-120.5204</v>
       </c>
       <c r="F7" s="51">
-        <f>[2]EB1!F12</f>
+        <f>'[2]EB1'!F12</f>
         <v>0</v>
       </c>
       <c r="G7" s="51">
-        <f>[2]EB1!G12</f>
+        <f>'[2]EB1'!G12</f>
         <v>-7.6189999999999998</v>
       </c>
       <c r="H7" s="51">
-        <f>[2]EB1!H12</f>
+        <f>'[2]EB1'!H12</f>
         <v>0</v>
       </c>
       <c r="I7" s="51">
-        <f>[2]EB1!I12</f>
+        <f>'[2]EB1'!I12</f>
         <v>-0.23350000000000001</v>
       </c>
       <c r="J7" s="51">
-        <f>[2]EB1!J12</f>
+        <f>'[2]EB1'!J12</f>
         <v>0</v>
       </c>
       <c r="K7" s="51">
-        <f>[2]EB1!K12</f>
+        <f>'[2]EB1'!K12</f>
         <v>0</v>
       </c>
       <c r="L7" s="51">
-        <f>[2]EB1!L12</f>
-        <v>-15.2</v>
+        <f>'[2]EB1'!L12</f>
+        <v>-15.199999999999999</v>
       </c>
       <c r="M7" s="51">
-        <f>[2]EB1!M12</f>
+        <f>'[2]EB1'!M12</f>
         <v>-1.772</v>
       </c>
       <c r="N7" s="51">
-        <f>[2]EB1!N12</f>
+        <f>'[2]EB1'!N12</f>
         <v>0</v>
       </c>
       <c r="O7" s="51">
-        <f>[2]EB1!O12</f>
+        <f>'[2]EB1'!O12</f>
         <v>-105.15525</v>
       </c>
       <c r="P7" s="51">
-        <f>[2]EB1!P12</f>
+        <f>'[2]EB1'!P12</f>
         <v>0</v>
       </c>
       <c r="Q7" s="51">
-        <f>[2]EB1!Q12</f>
+        <f>'[2]EB1'!Q12</f>
         <v>0</v>
       </c>
       <c r="R7" s="51">
-        <f>[2]EB1!R12</f>
+        <f>'[2]EB1'!R12</f>
         <v>0</v>
       </c>
       <c r="S7" s="51">
-        <f>[2]EB1!S12</f>
+        <f>'[2]EB1'!S12</f>
         <v>-0.78449999999999998</v>
       </c>
       <c r="T7" s="51">
-        <f>[2]EB1!T12</f>
+        <f>'[2]EB1'!T12</f>
         <v>329.37150000000003</v>
       </c>
       <c r="U7" s="51">
-        <f>[2]EB1!U12</f>
+        <f>'[2]EB1'!U12</f>
         <v>0</v>
       </c>
       <c r="V7" s="85">
-        <f>[2]EB1!V12</f>
+        <f>'[2]EB1'!V12</f>
         <v>-26.820549999999912</v>
       </c>
       <c r="X7" s="6"/>
     </row>
-    <row r="8" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="8" spans="2:22" ht="12.75">
       <c r="B8" s="50" t="s">
         <v>61</v>
       </c>
@@ -4792,83 +4755,83 @@
         <v>62</v>
       </c>
       <c r="D8" s="74">
-        <f>[2]EB1!D13</f>
+        <f>'[2]EB1'!D13</f>
         <v>0</v>
       </c>
       <c r="E8" s="51">
-        <f>[2]EB1!E13</f>
+        <f>'[2]EB1'!E13</f>
         <v>0</v>
       </c>
       <c r="F8" s="51">
-        <f>[2]EB1!F13</f>
+        <f>'[2]EB1'!F13</f>
         <v>-15868.2305</v>
       </c>
       <c r="G8" s="51">
-        <f>[2]EB1!G13</f>
-        <v>5701.34</v>
+        <f>'[2]EB1'!G13</f>
+        <v>5701.3400000000001</v>
       </c>
       <c r="H8" s="51">
-        <f>[2]EB1!H13</f>
+        <f>'[2]EB1'!H13</f>
         <v>969.47799999999995</v>
       </c>
       <c r="I8" s="51">
-        <f>[2]EB1!I13</f>
+        <f>'[2]EB1'!I13</f>
         <v>1086.3040000000001</v>
       </c>
       <c r="J8" s="51">
-        <f>[2]EB1!J13</f>
+        <f>'[2]EB1'!J13</f>
         <v>3354.9119999999998</v>
       </c>
       <c r="K8" s="51">
-        <f>[2]EB1!K13</f>
+        <f>'[2]EB1'!K13</f>
         <v>970.28800000000001</v>
       </c>
       <c r="L8" s="51">
-        <f>[2]EB1!L13</f>
+        <f>'[2]EB1'!L13</f>
         <v>2285.1019999999999</v>
       </c>
       <c r="M8" s="51">
-        <f>[2]EB1!M13</f>
+        <f>'[2]EB1'!M13</f>
         <v>1299.9449999999999</v>
       </c>
       <c r="N8" s="51">
-        <f>[2]EB1!N13</f>
+        <f>'[2]EB1'!N13</f>
         <v>0</v>
       </c>
       <c r="O8" s="51">
-        <f>[2]EB1!O13</f>
+        <f>'[2]EB1'!O13</f>
         <v>0</v>
       </c>
       <c r="P8" s="51">
-        <f>[2]EB1!P13</f>
+        <f>'[2]EB1'!P13</f>
         <v>0</v>
       </c>
       <c r="Q8" s="51">
-        <f>[2]EB1!Q13</f>
+        <f>'[2]EB1'!Q13</f>
         <v>0</v>
       </c>
       <c r="R8" s="51">
-        <f>[2]EB1!R13</f>
+        <f>'[2]EB1'!R13</f>
         <v>0</v>
       </c>
       <c r="S8" s="51">
-        <f>[2]EB1!S13</f>
+        <f>'[2]EB1'!S13</f>
         <v>0</v>
       </c>
       <c r="T8" s="51">
-        <f>[2]EB1!T13</f>
+        <f>'[2]EB1'!T13</f>
         <v>0</v>
       </c>
       <c r="U8" s="51">
-        <f>[2]EB1!U13</f>
+        <f>'[2]EB1'!U13</f>
         <v>0</v>
       </c>
       <c r="V8" s="85">
-        <f>[2]EB1!V13</f>
+        <f>'[2]EB1'!V13</f>
         <v>-200.86150000000021</v>
       </c>
     </row>
-    <row r="9" spans="1:27" ht="15" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:22" ht="15">
       <c r="B9" s="46"/>
       <c r="C9" s="55" t="s">
         <v>63</v>
@@ -4878,8 +4841,8 @@
         <v>-6381.1501000000017</v>
       </c>
       <c r="E9" s="56">
-        <f t="shared" ref="E9:U9" si="0">SUM(E5:E8)</f>
-        <v>-2691.93</v>
+        <f t="shared" si="0" ref="E9:U9">SUM(E5:E8)</f>
+        <v>-2691.9299999999998</v>
       </c>
       <c r="F9" s="56">
         <f t="shared" si="0"/>
@@ -4950,7 +4913,7 @@
         <v>-9781.6922875000037</v>
       </c>
     </row>
-    <row r="10" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:13" ht="12.75">
       <c r="A10" s="6"/>
       <c r="D10" s="10"/>
       <c r="F10" s="10"/>
@@ -4962,7 +4925,7 @@
       <c r="L10" s="10"/>
       <c r="M10" s="10"/>
     </row>
-    <row r="11" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:18" ht="12.75">
       <c r="A11" s="6"/>
       <c r="D11" s="10"/>
       <c r="E11" s="10"/>
@@ -4979,7 +4942,7 @@
       <c r="Q11" s="96"/>
       <c r="R11" s="96"/>
     </row>
-    <row r="12" spans="1:27" ht="15" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" ht="15">
       <c r="A12" s="6"/>
       <c r="C12" s="53" t="s">
         <v>142</v>
@@ -4995,15 +4958,15 @@
       <c r="L12" s="10"/>
       <c r="M12" s="10"/>
     </row>
-    <row r="13" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:22" ht="12.75">
       <c r="A13" s="6"/>
       <c r="V13" s="8"/>
     </row>
-    <row r="14" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:22" ht="12.75">
       <c r="A14" s="6"/>
       <c r="V14" s="8"/>
     </row>
-    <row r="15" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:22" ht="12.75">
       <c r="A15" s="6"/>
       <c r="C15" s="64" t="s">
         <v>89</v>
@@ -5016,7 +4979,7 @@
       </c>
       <c r="V15" s="8"/>
     </row>
-    <row r="16" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:22" ht="12.75">
       <c r="A16" s="6"/>
       <c r="B16" s="23" t="s">
         <v>98</v>
@@ -5032,7 +4995,7 @@
       </c>
       <c r="V16" s="8"/>
     </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="17" spans="2:5" ht="12.75">
       <c r="B17" s="50" t="s">
         <v>48</v>
       </c>
@@ -5044,33 +5007,33 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
+  <pageSetup orientation="portrait" paperSize="9" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="B1:M5"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
-    <col min="1" max="1" width="1.85546875" customWidth="1"/>
-    <col min="2" max="2" width="7.7109375" customWidth="1"/>
-    <col min="3" max="4" width="6.85546875" customWidth="1"/>
-    <col min="14" max="14" width="5.42578125" customWidth="1"/>
+    <col min="1" max="1" width="1.85714285714286" customWidth="1"/>
+    <col min="2" max="2" width="7.71428571428571" customWidth="1"/>
+    <col min="3" max="4" width="6.85714285714286" customWidth="1"/>
+    <col min="14" max="14" width="5.42857142857143" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="1" spans="5:6" ht="12.75">
       <c r="E1" s="11"/>
       <c r="F1" s="6"/>
     </row>
-    <row r="2" spans="2:13" ht="18" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:6" ht="18">
       <c r="B2" s="78" t="s">
         <v>146</v>
       </c>
       <c r="E2" s="6"/>
       <c r="F2" s="6"/>
     </row>
-    <row r="4" spans="2:13" ht="18" x14ac:dyDescent="0.25">
+    <row r="4" spans="5:13" ht="18">
       <c r="E4" s="119" t="s">
         <v>149</v>
       </c>
@@ -5083,7 +5046,7 @@
       <c r="L4" s="120"/>
       <c r="M4" s="121"/>
     </row>
-    <row r="5" spans="2:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="5:13" ht="12.75" customHeight="1">
       <c r="E5" s="79" t="s">
         <v>147</v>
       </c>
@@ -5101,37 +5064,37 @@
     <mergeCell ref="E4:M4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
-  <drawing r:id="rId2"/>
+  <pageSetup orientation="portrait" paperSize="9" r:id="rId2"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="B1:R33"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
-    <col min="2" max="2" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.5714285714286" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.1428571428571" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.8571428571429" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.5714285714286" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.28571428571429" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="9" customWidth="1"/>
-    <col min="9" max="9" width="2.140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.42578125" customWidth="1"/>
-    <col min="11" max="11" width="7.140625" customWidth="1"/>
-    <col min="12" max="12" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="61.7109375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="6.140625" customWidth="1"/>
-    <col min="15" max="15" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="8.140625" customWidth="1"/>
+    <col min="9" max="9" width="2.14285714285714" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.4285714285714" customWidth="1"/>
+    <col min="11" max="11" width="7.14285714285714" customWidth="1"/>
+    <col min="12" max="12" width="14.5714285714286" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="61.7142857142857" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="6.14285714285714" customWidth="1"/>
+    <col min="15" max="15" width="10.4285714285714" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="12.8571428571429" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="14.1428571428571" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="8.14285714285714" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:18" ht="15" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:8" ht="15">
       <c r="B1" s="12" t="s">
         <v>65</v>
       </c>
@@ -5152,7 +5115,7 @@
       </c>
       <c r="H1" s="39"/>
     </row>
-    <row r="2" spans="2:18" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:18" ht="31.5">
       <c r="B2" s="14" t="str">
         <f>'EB1'!B6</f>
         <v>ELC</v>
@@ -5188,7 +5151,7 @@
       <c r="Q2" s="107"/>
       <c r="R2" s="107"/>
     </row>
-    <row r="3" spans="2:18" x14ac:dyDescent="0.2">
+    <row r="3" spans="10:18" ht="12.75">
       <c r="J3" s="108" t="s">
         <v>7</v>
       </c>
@@ -5217,7 +5180,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="2:18" s="6" customFormat="1" ht="24" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:18" s="6" customFormat="1" ht="24" thickBot="1">
       <c r="B4" s="13"/>
       <c r="C4" s="13"/>
       <c r="D4" s="13"/>
@@ -5251,7 +5214,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="5" spans="2:18" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:18" ht="12.75">
       <c r="B5" s="8"/>
       <c r="C5" s="8"/>
       <c r="D5" s="8"/>
@@ -5272,7 +5235,7 @@
         <v>Electricity Plants Solid Fuels</v>
       </c>
       <c r="N5" s="111" t="str">
-        <f t="shared" ref="N5:N12" si="0">$E$2</f>
+        <f t="shared" si="0" ref="N5:N12">$E$2</f>
         <v>PJ</v>
       </c>
       <c r="O5" s="111"/>
@@ -5280,7 +5243,7 @@
       <c r="Q5" s="111"/>
       <c r="R5" s="111"/>
     </row>
-    <row r="6" spans="2:18" x14ac:dyDescent="0.2">
+    <row r="6" spans="2:18" ht="12.75">
       <c r="B6" s="8"/>
       <c r="C6" s="8"/>
       <c r="D6" s="8"/>
@@ -5307,7 +5270,7 @@
       <c r="Q6" s="111"/>
       <c r="R6" s="111"/>
     </row>
-    <row r="7" spans="2:18" x14ac:dyDescent="0.2">
+    <row r="7" spans="2:18" ht="12.75">
       <c r="B7" s="8"/>
       <c r="C7" s="8"/>
       <c r="D7" s="8"/>
@@ -5334,7 +5297,7 @@
       <c r="Q7" s="111"/>
       <c r="R7" s="111"/>
     </row>
-    <row r="8" spans="2:18" x14ac:dyDescent="0.2">
+    <row r="8" spans="2:18" ht="12.75">
       <c r="B8" s="8"/>
       <c r="C8" s="8"/>
       <c r="D8" s="8"/>
@@ -5361,7 +5324,7 @@
       <c r="Q8" s="111"/>
       <c r="R8" s="111"/>
     </row>
-    <row r="9" spans="2:18" x14ac:dyDescent="0.2">
+    <row r="9" spans="2:18" ht="12.75">
       <c r="B9" s="8"/>
       <c r="C9" s="8"/>
       <c r="D9" s="8"/>
@@ -5388,7 +5351,7 @@
       <c r="Q9" s="111"/>
       <c r="R9" s="111"/>
     </row>
-    <row r="10" spans="2:18" x14ac:dyDescent="0.2">
+    <row r="10" spans="2:18" ht="12.75">
       <c r="B10" s="8"/>
       <c r="C10" s="8"/>
       <c r="D10" s="8"/>
@@ -5415,7 +5378,7 @@
       <c r="Q10" s="111"/>
       <c r="R10" s="111"/>
     </row>
-    <row r="11" spans="2:18" x14ac:dyDescent="0.2">
+    <row r="11" spans="2:18" ht="12.75">
       <c r="B11" s="8"/>
       <c r="C11" s="8"/>
       <c r="D11" s="8"/>
@@ -5442,7 +5405,7 @@
       <c r="Q11" s="111"/>
       <c r="R11" s="111"/>
     </row>
-    <row r="12" spans="2:18" x14ac:dyDescent="0.2">
+    <row r="12" spans="2:18" ht="12.75">
       <c r="B12" s="8"/>
       <c r="C12" s="8"/>
       <c r="D12" s="8"/>
@@ -5469,11 +5432,11 @@
       <c r="Q12" s="111"/>
       <c r="R12" s="111"/>
     </row>
-    <row r="13" spans="2:18" x14ac:dyDescent="0.2">
+    <row r="13" spans="12:13" ht="12.75">
       <c r="L13" s="27"/>
       <c r="M13" s="29"/>
     </row>
-    <row r="14" spans="2:18" x14ac:dyDescent="0.2">
+    <row r="14" spans="4:18" ht="12.75">
       <c r="D14" s="4" t="s">
         <v>13</v>
       </c>
@@ -5491,7 +5454,7 @@
       <c r="Q14" s="113"/>
       <c r="R14" s="113"/>
     </row>
-    <row r="15" spans="2:18" x14ac:dyDescent="0.2">
+    <row r="15" spans="2:18" ht="12.75">
       <c r="B15" s="20" t="s">
         <v>1</v>
       </c>
@@ -5541,7 +5504,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="16" spans="2:18" ht="23.25" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:18" ht="23.25" thickBot="1">
       <c r="B16" s="19" t="s">
         <v>37</v>
       </c>
@@ -5591,7 +5554,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="17" spans="2:18" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:18" ht="13.5" thickBot="1">
       <c r="B17" s="18" t="s">
         <v>76</v>
       </c>
@@ -5618,7 +5581,7 @@
       <c r="Q17" s="114"/>
       <c r="R17" s="114"/>
     </row>
-    <row r="18" spans="2:18" x14ac:dyDescent="0.2">
+    <row r="18" spans="2:18" ht="12.75">
       <c r="B18" s="25" t="str">
         <f>Sector_Fuels_ELC!L18</f>
         <v>FTE-ELCCOA</v>
@@ -5644,26 +5607,26 @@
       </c>
       <c r="K18" s="116"/>
       <c r="L18" s="111" t="str">
-        <f t="shared" ref="L18:L25" si="1">"FT"&amp;$G$2&amp;"-"&amp;L5</f>
+        <f t="shared" si="1" ref="L18:L25">"FT"&amp;$G$2&amp;"-"&amp;L5</f>
         <v>FTE-ELCCOA</v>
       </c>
       <c r="M18" s="112" t="str">
-        <f t="shared" ref="M18:M25" si="2">$D$2&amp;" Technology"&amp;" "&amp;$G$1&amp;" "&amp;M5</f>
+        <f t="shared" si="2" ref="M18:M25">$D$2&amp;" Technology"&amp;" "&amp;$G$1&amp;" "&amp;M5</f>
         <v>Sector Fuel Technology Existing Electricity Plants Solid Fuels</v>
       </c>
       <c r="N18" s="111" t="str">
-        <f t="shared" ref="N18:N25" si="3">$E$2</f>
+        <f t="shared" si="3" ref="N18:N25">$E$2</f>
         <v>PJ</v>
       </c>
       <c r="O18" s="111" t="str">
-        <f t="shared" ref="O18:O25" si="4">$E$2&amp;"a"</f>
+        <f t="shared" si="4" ref="O18:O25">$E$2&amp;"a"</f>
         <v>PJa</v>
       </c>
       <c r="P18" s="111"/>
       <c r="Q18" s="111"/>
       <c r="R18" s="111"/>
     </row>
-    <row r="19" spans="2:18" x14ac:dyDescent="0.2">
+    <row r="19" spans="2:18" ht="12.75">
       <c r="B19" s="25" t="str">
         <f>Sector_Fuels_ELC!L19</f>
         <v>FTE-ELCGAS</v>
@@ -5706,7 +5669,7 @@
       <c r="Q19" s="111"/>
       <c r="R19" s="111"/>
     </row>
-    <row r="20" spans="2:18" x14ac:dyDescent="0.2">
+    <row r="20" spans="2:18" ht="12.75">
       <c r="B20" s="25" t="str">
         <f>Sector_Fuels_ELC!L20</f>
         <v>FTE-ELCOIL</v>
@@ -5721,7 +5684,7 @@
       </c>
       <c r="E20" s="70">
         <f>-'EB1'!G$6/-SUM('EB1'!$G$6:$M$6)</f>
-        <v>4.9257354796510562E-2</v>
+        <v>0.049257354796510562</v>
       </c>
       <c r="F20" s="16"/>
       <c r="G20" s="71">
@@ -5752,7 +5715,7 @@
       <c r="Q20" s="111"/>
       <c r="R20" s="111"/>
     </row>
-    <row r="21" spans="2:18" x14ac:dyDescent="0.2">
+    <row r="21" spans="2:18" ht="12.75">
       <c r="B21" s="25"/>
       <c r="C21" t="str">
         <f>'EB1'!I$2</f>
@@ -5761,7 +5724,7 @@
       <c r="D21" s="25"/>
       <c r="E21" s="70">
         <f>-'EB1'!I$6/-SUM('EB1'!$G$6:$M$6)</f>
-        <v>3.8926710484734312E-2</v>
+        <v>0.038926710484734312</v>
       </c>
       <c r="F21" s="16"/>
       <c r="G21" s="71"/>
@@ -5788,7 +5751,7 @@
       <c r="Q21" s="117"/>
       <c r="R21" s="111"/>
     </row>
-    <row r="22" spans="2:18" x14ac:dyDescent="0.2">
+    <row r="22" spans="2:18" ht="12.75">
       <c r="B22" s="25"/>
       <c r="C22" t="str">
         <f>'EB1'!L$2</f>
@@ -5824,7 +5787,7 @@
       <c r="Q22" s="111"/>
       <c r="R22" s="111"/>
     </row>
-    <row r="23" spans="2:18" x14ac:dyDescent="0.2">
+    <row r="23" spans="2:18" ht="12.75">
       <c r="B23" s="25"/>
       <c r="C23" t="str">
         <f>'EB1'!M$2</f>
@@ -5833,7 +5796,7 @@
       <c r="D23" s="25"/>
       <c r="E23" s="70">
         <f>-'EB1'!M$6/-SUM('EB1'!$G$6:$M$6)</f>
-        <v>5.4758702573637796E-2</v>
+        <v>0.054758702573637796</v>
       </c>
       <c r="F23" s="16"/>
       <c r="G23" s="71"/>
@@ -5860,7 +5823,7 @@
       <c r="Q23" s="113"/>
       <c r="R23" s="113"/>
     </row>
-    <row r="24" spans="2:18" x14ac:dyDescent="0.2">
+    <row r="24" spans="2:18" ht="12.75">
       <c r="B24" s="28" t="str">
         <f>Sector_Fuels_ELC!L21</f>
         <v>FTE-ELCNUC</v>
@@ -5903,7 +5866,7 @@
       <c r="Q24" s="113"/>
       <c r="R24" s="113"/>
     </row>
-    <row r="25" spans="2:18" x14ac:dyDescent="0.2">
+    <row r="25" spans="2:18" ht="12.75">
       <c r="B25" s="28" t="str">
         <f>Sector_Fuels_ELC!L22</f>
         <v>FTE-ELCBIO</v>
@@ -5946,7 +5909,7 @@
       <c r="Q25" s="113"/>
       <c r="R25" s="113"/>
     </row>
-    <row r="26" spans="2:18" x14ac:dyDescent="0.2">
+    <row r="26" spans="2:8" ht="12.75">
       <c r="B26" s="28" t="str">
         <f>Sector_Fuels_ELC!L23</f>
         <v>FTE-ELCHYD</v>
@@ -5968,7 +5931,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="27" spans="2:18" x14ac:dyDescent="0.2">
+    <row r="27" spans="2:8" ht="12.75">
       <c r="B27" s="28" t="str">
         <f>Sector_Fuels_ELC!L24</f>
         <v>FTE-ELCWIN</v>
@@ -5990,7 +5953,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="28" spans="2:18" x14ac:dyDescent="0.2">
+    <row r="28" spans="2:8" ht="12.75">
       <c r="B28" s="28" t="str">
         <f>Sector_Fuels_ELC!L25</f>
         <v>FTE-ELCSOL</v>
@@ -6012,13 +5975,13 @@
         <v>30</v>
       </c>
     </row>
-    <row r="32" spans="2:18" x14ac:dyDescent="0.2">
+    <row r="32" spans="2:3" ht="12.75">
       <c r="B32" s="52"/>
       <c r="C32" s="1" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="33" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="33" spans="2:3" ht="12.75">
       <c r="B33" s="68"/>
       <c r="C33" s="1" t="s">
         <v>145</v>
@@ -6026,46 +5989,46 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait" paperSize="9" r:id="rId4"/>
   <drawing r:id="rId2"/>
   <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="B1:AB65536"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85428571428571" defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" width="3" style="25" customWidth="1"/>
-    <col min="2" max="2" width="16.42578125" style="25" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" style="25" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.28515625" style="25" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.4285714285714" style="25" customWidth="1"/>
+    <col min="3" max="3" width="12.1428571428571" style="25" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.2857142857143" style="25" bestFit="1" customWidth="1"/>
     <col min="5" max="6" width="12" style="25" bestFit="1" customWidth="1"/>
     <col min="7" max="8" width="13" style="25" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.85546875" style="25" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.140625" style="25" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.85714285714286" style="25" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.14285714285714" style="25" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="10" style="25" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9.85546875" style="25" bestFit="1" customWidth="1"/>
-    <col min="13" max="14" width="8.85546875" style="25" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.85714285714286" style="25" bestFit="1" customWidth="1"/>
+    <col min="13" max="14" width="8.85714285714286" style="25" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="15" style="25" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="13.28515625" style="25" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.2857142857143" style="25" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="2" style="25" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="13.5703125" style="25" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="2.140625" style="27" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="7.42578125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="43.28515625" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="6.28515625" customWidth="1"/>
-    <col min="25" max="25" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="13.5714285714286" style="25" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="2.14285714285714" style="27" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="12.4285714285714" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="7.42857142857143" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="14.5714285714286" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="43.2857142857143" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="6.28571428571429" customWidth="1"/>
+    <col min="25" max="25" width="11.4285714285714" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="13.5714285714286" bestFit="1" customWidth="1"/>
     <col min="27" max="27" width="15" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="8.140625" bestFit="1" customWidth="1"/>
-    <col min="29" max="16384" width="8.85546875" style="25"/>
+    <col min="28" max="28" width="8.14285714285714" bestFit="1" customWidth="1"/>
+    <col min="29" max="16384" width="8.85714285714286" style="25"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:28" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:8" ht="30">
       <c r="B1" s="24" t="s">
         <v>65</v>
       </c>
@@ -6088,7 +6051,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="2" spans="2:28" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:28" ht="31.5">
       <c r="B2" s="14" t="str">
         <f>'EB1'!B6</f>
         <v>ELC</v>
@@ -6126,7 +6089,7 @@
       <c r="AA2" s="107"/>
       <c r="AB2" s="107"/>
     </row>
-    <row r="3" spans="2:28" x14ac:dyDescent="0.2">
+    <row r="3" spans="20:28" ht="12.75">
       <c r="T3" s="108" t="s">
         <v>7</v>
       </c>
@@ -6155,7 +6118,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="2:28" s="26" customFormat="1" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:28" s="26" customFormat="1" ht="30.75" thickBot="1">
       <c r="B4" s="33" t="s">
         <v>107</v>
       </c>
@@ -6202,7 +6165,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="5" spans="2:28" s="26" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:28" s="26" customFormat="1" ht="15.75">
       <c r="B5" s="32" t="s">
         <v>113</v>
       </c>
@@ -6246,7 +6209,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="6" spans="2:28" x14ac:dyDescent="0.2">
+    <row r="6" spans="20:28" ht="12.75">
       <c r="T6" s="113" t="s">
         <v>88</v>
       </c>
@@ -6268,11 +6231,11 @@
       <c r="AA6" s="113"/>
       <c r="AB6" s="113"/>
     </row>
-    <row r="7" spans="2:28" x14ac:dyDescent="0.2">
+    <row r="7" spans="20:21" ht="12.75">
       <c r="T7" s="2"/>
       <c r="U7" s="2"/>
     </row>
-    <row r="8" spans="2:28" x14ac:dyDescent="0.2">
+    <row r="8" spans="4:28" ht="12.75">
       <c r="D8" s="4" t="s">
         <v>13</v>
       </c>
@@ -6297,7 +6260,7 @@
       <c r="AA8" s="107"/>
       <c r="AB8" s="107"/>
     </row>
-    <row r="9" spans="2:28" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="2:28" ht="12.75" customHeight="1">
       <c r="B9" s="21" t="s">
         <v>1</v>
       </c>
@@ -6376,7 +6339,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="2:28" ht="23.25" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:28" ht="23.25" thickBot="1">
       <c r="B10" s="19" t="s">
         <v>37</v>
       </c>
@@ -6455,7 +6418,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="2:28" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:28" ht="13.5" thickBot="1">
       <c r="B11" s="18" t="s">
         <v>76</v>
       </c>
@@ -6516,9 +6479,9 @@
       <c r="AA11" s="110"/>
       <c r="AB11" s="110"/>
     </row>
-    <row r="12" spans="2:28" x14ac:dyDescent="0.2">
+    <row r="12" spans="2:28" ht="12.75">
       <c r="B12" s="25" t="str">
-        <f t="shared" ref="B12:B19" si="0">V12</f>
+        <f t="shared" si="0" ref="B12:B19">V12</f>
         <v>ELCTECOA00</v>
       </c>
       <c r="C12" s="25" t="str">
@@ -6526,7 +6489,7 @@
         <v>ELCCOA</v>
       </c>
       <c r="D12" s="25" t="str">
-        <f t="shared" ref="D12:D19" si="1">$V$5</f>
+        <f t="shared" si="1" ref="D12:D19">$V$5</f>
         <v>ELC</v>
       </c>
       <c r="G12" s="98">
@@ -6545,7 +6508,7 @@
         <v>40</v>
       </c>
       <c r="M12" s="76">
-        <v>0.5</v>
+        <v>0.50</v>
       </c>
       <c r="N12" s="75">
         <v>30</v>
@@ -6558,7 +6521,7 @@
       </c>
       <c r="Q12" s="26"/>
       <c r="R12" s="34">
-        <f t="shared" ref="R12:R19" si="2">G12*$J12*$O12</f>
+        <f t="shared" si="2" ref="R12:R19">G12*$J12*$O12</f>
         <v>2395.6907520000004</v>
       </c>
       <c r="S12" s="100"/>
@@ -6575,11 +6538,11 @@
         <v>Power Plants Existing00 - Solid Fuels</v>
       </c>
       <c r="X12" s="111" t="str">
-        <f t="shared" ref="X12:X19" si="3">$E$2</f>
+        <f t="shared" si="3" ref="X12:X19">$E$2</f>
         <v>PJ</v>
       </c>
       <c r="Y12" s="111" t="str">
-        <f t="shared" ref="Y12:Y19" si="4">$F$2</f>
+        <f t="shared" si="4" ref="Y12:Y19">$F$2</f>
         <v>GW</v>
       </c>
       <c r="Z12" s="115" t="s">
@@ -6588,7 +6551,7 @@
       <c r="AA12" s="111"/>
       <c r="AB12" s="111"/>
     </row>
-    <row r="13" spans="2:28" x14ac:dyDescent="0.2">
+    <row r="13" spans="2:28" ht="12.75">
       <c r="B13" s="25" t="str">
         <f t="shared" si="0"/>
         <v>ELCTEGAS00</v>
@@ -6617,7 +6580,7 @@
         <v>35</v>
       </c>
       <c r="M13" s="76">
-        <v>0.4</v>
+        <v>0.40</v>
       </c>
       <c r="N13" s="75">
         <v>20</v>
@@ -6656,7 +6619,7 @@
       <c r="AA13" s="111"/>
       <c r="AB13" s="111"/>
     </row>
-    <row r="14" spans="2:28" x14ac:dyDescent="0.2">
+    <row r="14" spans="2:28" ht="12.75">
       <c r="B14" s="25" t="str">
         <f t="shared" si="0"/>
         <v>ELCTEOIL00</v>
@@ -6685,7 +6648,7 @@
         <v>20</v>
       </c>
       <c r="M14" s="94">
-        <v>0.2</v>
+        <v>0.20</v>
       </c>
       <c r="N14" s="93">
         <v>30</v>
@@ -6724,7 +6687,7 @@
       <c r="AA14" s="111"/>
       <c r="AB14" s="111"/>
     </row>
-    <row r="15" spans="2:28" x14ac:dyDescent="0.2">
+    <row r="15" spans="2:28" ht="12.75">
       <c r="B15" s="28" t="str">
         <f t="shared" si="0"/>
         <v>ELCNENUC00</v>
@@ -6751,7 +6714,7 @@
         <v>0.33</v>
       </c>
       <c r="J15" s="94">
-        <v>0.9</v>
+        <v>0.90</v>
       </c>
       <c r="K15" s="93"/>
       <c r="L15" s="94">
@@ -6797,7 +6760,7 @@
       <c r="AA15" s="111"/>
       <c r="AB15" s="111"/>
     </row>
-    <row r="16" spans="2:28" x14ac:dyDescent="0.2">
+    <row r="16" spans="2:28" ht="12.75">
       <c r="B16" s="28" t="str">
         <f t="shared" si="0"/>
         <v>ELCREBIO00</v>
@@ -6821,7 +6784,7 @@
         <v>0.28000000000000003</v>
       </c>
       <c r="J16" s="73">
-        <v>0.6</v>
+        <v>0.60</v>
       </c>
       <c r="K16" s="73"/>
       <c r="L16" s="74">
@@ -6867,7 +6830,7 @@
       <c r="AA16" s="111"/>
       <c r="AB16" s="111"/>
     </row>
-    <row r="17" spans="2:28" x14ac:dyDescent="0.2">
+    <row r="17" spans="2:28" ht="12.75">
       <c r="B17" s="28" t="str">
         <f t="shared" si="0"/>
         <v>ELCREHYD00</v>
@@ -6892,7 +6855,7 @@
         <v>1</v>
       </c>
       <c r="J17" s="73">
-        <v>0.5</v>
+        <v>0.50</v>
       </c>
       <c r="K17" s="73"/>
       <c r="L17" s="74">
@@ -6908,7 +6871,7 @@
         <v>31.536000000000001</v>
       </c>
       <c r="P17" s="94">
-        <v>0.5</v>
+        <v>0.50</v>
       </c>
       <c r="Q17" s="28"/>
       <c r="R17" s="34">
@@ -6938,7 +6901,7 @@
       <c r="AA17" s="111"/>
       <c r="AB17" s="111"/>
     </row>
-    <row r="18" spans="2:28" x14ac:dyDescent="0.2">
+    <row r="18" spans="2:28" ht="12.75">
       <c r="B18" s="28" t="str">
         <f t="shared" si="0"/>
         <v>ELCREWIN00</v>
@@ -6969,7 +6932,7 @@
         <v>35</v>
       </c>
       <c r="M18" s="73">
-        <v>0.5</v>
+        <v>0.50</v>
       </c>
       <c r="N18" s="74">
         <v>20</v>
@@ -6978,7 +6941,7 @@
         <v>31.536000000000001</v>
       </c>
       <c r="P18" s="94">
-        <v>0.3</v>
+        <v>0.30</v>
       </c>
       <c r="Q18" s="28"/>
       <c r="R18" s="34">
@@ -7008,7 +6971,7 @@
       <c r="AA18" s="111"/>
       <c r="AB18" s="111"/>
     </row>
-    <row r="19" spans="2:28" x14ac:dyDescent="0.2">
+    <row r="19" spans="2:28" ht="12.75">
       <c r="B19" s="28" t="str">
         <f t="shared" si="0"/>
         <v>ELCRESOL00</v>
@@ -7032,7 +6995,7 @@
         <v>1</v>
       </c>
       <c r="J19" s="73">
-        <v>0.3</v>
+        <v>0.30</v>
       </c>
       <c r="K19" s="73"/>
       <c r="L19" s="74">
@@ -7046,7 +7009,7 @@
         <v>31.536000000000001</v>
       </c>
       <c r="P19" s="94">
-        <v>0.2</v>
+        <v>0.20</v>
       </c>
       <c r="Q19" s="28"/>
       <c r="R19" s="34">
@@ -7076,49 +7039,49 @@
       <c r="AA19" s="111"/>
       <c r="AB19" s="111"/>
     </row>
-    <row r="21" spans="2:28" x14ac:dyDescent="0.2">
+    <row r="21" spans="18:18" ht="12.75">
       <c r="R21" s="97"/>
     </row>
-    <row r="22" spans="2:28" x14ac:dyDescent="0.2">
+    <row r="22" spans="18:18" ht="12.75">
       <c r="R22" s="97"/>
     </row>
-    <row r="23" spans="2:28" x14ac:dyDescent="0.2">
+    <row r="23" spans="2:18" ht="12.75">
       <c r="B23" s="52"/>
       <c r="C23" s="1" t="s">
         <v>144</v>
       </c>
       <c r="R23" s="97"/>
     </row>
-    <row r="24" spans="2:28" x14ac:dyDescent="0.2">
+    <row r="24" spans="2:18" ht="12.75">
       <c r="B24" s="68"/>
       <c r="C24" s="1" t="s">
         <v>145</v>
       </c>
       <c r="R24" s="97"/>
     </row>
-    <row r="25" spans="2:28" x14ac:dyDescent="0.2">
+    <row r="25" spans="18:18" ht="12.75">
       <c r="R25" s="97"/>
     </row>
-    <row r="65536" spans="19:19" x14ac:dyDescent="0.2">
+    <row r="65536" spans="19:19" ht="12.75">
       <c r="S65536" s="37"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
+  <pageSetup orientation="portrait" paperSize="9" r:id="rId4"/>
   <drawing r:id="rId2"/>
   <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="B3:J24"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
-    <col min="2" max="2" width="14.42578125" customWidth="1"/>
+    <col min="2" max="2" width="14.4285714285714" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:10" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:10" ht="17.45" customHeight="1">
       <c r="B3" s="42" t="s">
         <v>150</v>
       </c>
@@ -7131,7 +7094,7 @@
       <c r="I3" s="42"/>
       <c r="J3" s="42"/>
     </row>
-    <row r="4" spans="2:10" s="6" customFormat="1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:7" s="6" customFormat="1" ht="17.45" customHeight="1">
       <c r="B4" s="43"/>
       <c r="C4" s="43"/>
       <c r="D4" s="43"/>
@@ -7139,7 +7102,7 @@
       <c r="F4" s="43"/>
       <c r="G4" s="43"/>
     </row>
-    <row r="5" spans="2:10" ht="18" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:7" ht="18">
       <c r="B5" s="40" t="s">
         <v>138</v>
       </c>
@@ -7147,7 +7110,7 @@
       <c r="F5" s="31"/>
       <c r="G5" s="31"/>
     </row>
-    <row r="6" spans="2:10" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:8" ht="13.5" thickBot="1">
       <c r="B6" s="45" t="s">
         <v>0</v>
       </c>
@@ -7167,7 +7130,7 @@
       <c r="G6" s="44"/>
       <c r="H6" s="1"/>
     </row>
-    <row r="7" spans="2:10" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:8" ht="13.5" thickBot="1">
       <c r="B7" s="18" t="s">
         <v>76</v>
       </c>
@@ -7184,7 +7147,7 @@
       <c r="G7" s="88"/>
       <c r="H7" s="1"/>
     </row>
-    <row r="8" spans="2:10" x14ac:dyDescent="0.2">
+    <row r="8" spans="2:8" ht="12.75">
       <c r="B8" s="25" t="str">
         <f>Con_ELC!$V$6</f>
         <v>ELCCO2</v>
@@ -7193,7 +7156,7 @@
         <v>95</v>
       </c>
       <c r="D8" s="73">
-        <v>56.1</v>
+        <v>56.10</v>
       </c>
       <c r="E8" s="73">
         <v>76.400000000000006</v>
@@ -7202,21 +7165,21 @@
       <c r="G8" s="89"/>
       <c r="H8" s="1"/>
     </row>
-    <row r="9" spans="2:10" x14ac:dyDescent="0.2">
+    <row r="9" spans="6:7" ht="12.75">
       <c r="F9" s="31"/>
       <c r="G9" s="31"/>
     </row>
-    <row r="10" spans="2:10" x14ac:dyDescent="0.2">
+    <row r="10" spans="6:7" ht="12.75">
       <c r="F10" s="31"/>
       <c r="G10" s="31"/>
     </row>
-    <row r="23" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="23" spans="2:3" ht="12.75">
       <c r="B23" s="52"/>
       <c r="C23" s="1" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="24" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="24" spans="2:3" ht="12.75">
       <c r="B24" s="68"/>
       <c r="C24" s="1" t="s">
         <v>145</v>

</xml_diff>